<commit_message>
feat(productos): Kit de Tareas Heladería v2.0 (298 tareas) y Hotel v2.0 (636 tareas, 19 ficheros) — motor 2.4 + contenido propio; molde P4 normalizado; idempotencia 0, censo 0, gate offline 11/11 y 19/19
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-heladeria/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas-heladeria/01-apertura-cierre.xlsx
@@ -90,7 +90,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -151,6 +151,11 @@
         <bgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -178,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -229,6 +234,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -638,7 +646,7 @@
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>▸ Incluye encendido de vitrinas, cámaras, montaje de servicio y cierre.</t>
+          <t>▸ Incluye el paso de las vitrinas a modo servicio, la comprobación de cámaras, el montaje y el cierre.</t>
         </is>
       </c>
     </row>
@@ -680,9 +688,45 @@
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-heladeria · info@aichef.pro</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Higiene, alérgenos y temperaturas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>▸ La primera sección de «Apertura» es de higiene personal y de arranque seguro: extracción primero y, si tienes gas para gofres o crepes, comprobación de olor antes de encender nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>▸ Las tres temperaturas de una heladería son distintas y no se mezclan: conservación −18 °C, servicio de vitrina −14 a −12 °C y maduración de la mezcla 2-4 °C. Las vitrinas NO se apagan por la noche: pasan a conservación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>▸ Los alérgenos viajan en la pala: un porcionador por cubeta y enjuague entre sabores. El barquillo y la galleta llevan gluten, y pistacho, avellana y almendra son de declaración obligatoria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-tareas-heladeria · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -707,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -737,7 +781,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Encendido y verificación de equipos</t>
+          <t>Higiene personal y arranque seguro</t>
         </is>
       </c>
     </row>
@@ -784,12 +828,12 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Encender vitrinas de exposición y verificar temperatura -14°C/-12°C</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Vitrina</t>
+          <t>Uniforme y delantal limpios, pelo recogido con gorro o redecilla y calzado antideslizante</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
         </is>
       </c>
       <c r="D6" s="11" t="n"/>
@@ -803,12 +847,12 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Verificar cámaras de conservación a -18°C</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Cámara</t>
+          <t>Sin anillos, reloj ni pulseras; uñas cortas, limpias y sin esmalte: se sirve con porcionador y se manipulan cucuruchos y toppings</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
         </is>
       </c>
       <c r="D7" s="11" t="n"/>
@@ -822,12 +866,12 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Verificar cámara de maduración a 2-4°C</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>Maduración</t>
+          <t>Heridas y cortes cubiertos con apósito impermeable de color visible y guante encima</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
         </is>
       </c>
       <c r="D8" s="11" t="n"/>
@@ -841,12 +885,12 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Comprobar abatidor de temperatura operativo</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Abatidor</t>
+          <t>Lavado de manos al entrar y en cada cambio de tarea: jabón, agua caliente y papel de un solo uso</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
         </is>
       </c>
       <c r="D9" s="11" t="n"/>
@@ -860,12 +904,12 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Encender iluminación de vitrinas y sala</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Vitrina</t>
+          <t>Declarar síntomas digestivos o respiratorios: quien los tenga no manipula helado, fruta ni toppings</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
         </is>
       </c>
       <c r="D10" s="11" t="n"/>
@@ -879,12 +923,12 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Registrar temperaturas en hoja de control APPCC</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>Admin</t>
+          <t>Encender la extracción del obrador y ventilar antes de poner en marcha pasteurizador y mantecadora</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Obrador</t>
         </is>
       </c>
       <c r="D11" s="11" t="n"/>
@@ -892,82 +936,84 @@
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="13" t="n"/>
     </row>
-    <row r="12"/>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Si el obrador o la zona de gofres/crepes tiene GAS: abrir la llave general y comprobar que NO huele a gas ANTES de encender nada. Si huele, no enciendas, ventila y avisa al mantenedor</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Obrador</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="13" t="n"/>
+    </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Montaje de servicio</t>
-        </is>
-      </c>
+      <c r="A13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Encendido y verificación de equipos</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Montar toppings frescos: fruta, frutos secos, virutas de chocolate</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>Mostrador</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Preparar salsas: chocolate, caramelo, frutos rojos, dulce de leche</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>Mostrador</t>
+          <t>Pasar las vitrinas de exposición de conservación nocturna (−18 °C) a modo servicio (−14 a −12 °C) y comprobar que han mantenido la temperatura toda la noche — anota la lectura: ____ °C</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Vitrina</t>
         </is>
       </c>
       <c r="D16" s="11" t="n"/>
@@ -977,16 +1023,16 @@
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Reponer cucuruchos, tarrinas, cucharillas y servilletas</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>Mostrador</t>
+          <t>Comprobar que las cámaras de conservación han funcionado toda la noche y registrar la temperatura (≤ −18 °C) — anota la lectura: ____ °C. Si hay desviación, no sirvas el producto hasta valorarlo</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="D17" s="11" t="n"/>
@@ -996,16 +1042,16 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Verificar stock de conos artesanales y barquillos</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>Mostrador</t>
+          <t>Comprobar la cámara de maduración (2-4 °C) — anota la lectura: ____ °C: por encima de 4 °C una mezcla pasteurizada vuelve a ser un caldo de cultivo</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Maduración</t>
         </is>
       </c>
       <c r="D18" s="11" t="n"/>
@@ -1015,16 +1061,16 @@
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Limpiar cristales de vitrina (interior y exterior)</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>Limpieza</t>
+          <t>Comprobar abatidor de temperatura operativo</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Abatidor</t>
         </is>
       </c>
       <c r="D19" s="11" t="n"/>
@@ -1034,11 +1080,11 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Verificar aspecto visual de cubetas en vitrina (sin cristales de hielo)</t>
+          <t>Encender iluminación de vitrinas y sala</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -1051,82 +1097,82 @@
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="13" t="n"/>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Apertura al público</t>
-        </is>
-      </c>
-    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Registrar las temperaturas del día (vitrinas, cámaras y maduración): si tienes el Pack APPCC, en su hoja de temperaturas; si no, en la columna «Notas» de esta hoja</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="13" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Montaje de servicio</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Encender TPV / caja registradora y verificar fondo de caja</t>
-        </is>
-      </c>
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>Caja</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Verificar datáfono y terminal de pagos operativo</t>
+          <t>Montar toppings frescos: la FRUTA que se sirve cruda, lavada y desinfectada con lejía apta para uso alimentario según la dosis del fabricante (habitual: 70 ppm, 5 min) y ACLARADA con agua potable abundante; frutos secos y virutas, en recipiente cerrado</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>Caja</t>
+          <t>Mostrador</t>
         </is>
       </c>
       <c r="D25" s="11" t="n"/>
@@ -1136,11 +1182,11 @@
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Colocar pizarra/carta exterior con sabores del día</t>
+          <t>Un porcionador por cubeta y enjuague entre sabores: el pistacho, la avellana y la almendra viajan de una cubeta a otra en la pala y son ALÉRGENOS de declaración obligatoria</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
@@ -1155,16 +1201,16 @@
     </row>
     <row r="27">
       <c r="A27" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Verificar limpieza de zona de terraza/exterior si procede</t>
-        </is>
-      </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>Terraza</t>
+          <t>Tener a la vista la carta de ALÉRGENOS por sabor y comprobar que se corresponde con las cubetas que hay hoy en vitrina (leche, frutos secos, huevo, gluten del barquillo y la galleta, soja y sulfitos)</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Mostrador</t>
         </is>
       </c>
       <c r="D27" s="11" t="n"/>
@@ -1174,16 +1220,16 @@
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Abrir puerta y encender rótulo exterior</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="inlineStr">
-        <is>
-          <t>General</t>
+          <t>Preparar salsas: chocolate, caramelo, frutos rojos, dulce de leche</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Mostrador</t>
         </is>
       </c>
       <c r="D28" s="11" t="n"/>
@@ -1192,57 +1238,274 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="21" t="inlineStr">
+      <c r="A29" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Reponer cucuruchos, tarrinas, cucharillas y servilletas</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Mostrador</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="13" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Verificar stock de conos artesanales y barquillos</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Mostrador</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Limpiar cristales de vitrina (interior y exterior)</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Limpieza</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="13" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Verificar aspecto visual de cubetas en vitrina (sin cristales de hielo)</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Vitrina</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="13" t="n"/>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Apertura al público</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Encender TPV / caja registradora y verificar fondo de caja</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="13" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Verificar datáfono y terminal de pagos operativo</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="13" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Colocar pizarra/carta exterior con sabores del día</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Mostrador</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Verificar limpieza de zona de terraza/exterior si procede</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>Terraza</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Abrir puerta y encender rótulo exterior</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>Tareas completadas:</t>
         </is>
       </c>
-      <c r="C29">
-        <f>COUNTIF(E6:E28,"✓")</f>
-        <v>2.0</v>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="C41">
+        <f>COUNTIFS(B6:B40,"?*",E6:E40,"✓")-COUNTIFS(B6:B40,"Tarea",E6:E40,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="E29">
-        <f>COUNTIF(B6:B28,"?*")</f>
-        <v>19.0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="E41">
+        <f>COUNTIF(B6:B40,"?*")-COUNTIF(B6:B40,"Tarea")-COUNTIF(E6:E40,"N/A")</f>
+        <v>26.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Firma responsable: _________________  Fecha: ___/___/______</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A42:G42"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:G28">
+  <conditionalFormatting sqref="A6:G40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E6="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E15 E16 E17 E18 E19 E20 E24 E25 E26 E27 E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa ✓, ✗ o —" prompt="Marca ✓ si completada" type="list">
-      <formula1>"✓,✗,—"</formula1>
+    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E12 E16 E17 E18 E19 E20 E21 E25 E26 E27 E28 E29 E30 E31 E32 E36 E37 E38 E39 E40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." prompt="Marca ✓ si completada" type="list" errorStyle="stop">
+      <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -1361,7 +1624,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Pasar vitrinas a modo conservación -18°C</t>
+          <t>Pasar las vitrinas de exposición a modo conservación (−18 °C): no se apagan — con género dentro, una parada nocturna se lleva por delante la partida entera</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -1380,7 +1643,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Registrar mermas del día (sabores agotados, producto desechado)</t>
+          <t>Anotar las mermas del día (sabor, kg y motivo: agotado, desechado, cristalizado o descongelado): es el dato que corrige el food cost y la planificación de producción de mañana</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -1756,8 +2019,8 @@
         </is>
       </c>
       <c r="C29">
-        <f>COUNTIF(E6:E28,"✓")</f>
-        <v>2.0</v>
+        <f>COUNTIFS(B6:B28,"?*",E6:E28,"✓")-COUNTIFS(B6:B28,"Tarea",E6:E28,"✓")</f>
+        <v>0.0</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1765,8 +2028,8 @@
         </is>
       </c>
       <c r="E29">
-        <f>COUNTIF(B6:B28,"?*")</f>
-        <v>19.0</v>
+        <f>COUNTIF(B6:B28,"?*")-COUNTIF(B6:B28,"Tarea")-COUNTIF(E6:E28,"N/A")</f>
+        <v>17.0</v>
       </c>
     </row>
     <row r="30">
@@ -1799,8 +2062,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E6 E7 E8 E9 E10 E14 E15 E16 E17 E18 E19 E20 E24 E25 E26 E27 E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa ✓, ✗ o —" prompt="Marca ✓ si completada" type="list">
-      <formula1>"✓,✗,—"</formula1>
+    <dataValidation sqref="E6 E7 E8 E9 E10 E14 E15 E16 E17 E18 E19 E20 E24 E25 E26 E27 E28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." prompt="Marca ✓ si completada" type="list" errorStyle="stop">
+      <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>

</xml_diff>